<commit_message>
applied same capacity demand - that accounts for simultaneity - for both FBMC and NTC
</commit_message>
<xml_diff>
--- a/analysis_data/getting_parameters.xlsx
+++ b/analysis_data/getting_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kadekola\github_codes\cross_border-CM\analysis_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4FF5EC-16BE-4AFE-8545-94C202A51FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F341F13-E6D2-44E4-AC76-D3D137832BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="5" r:id="rId1"/>
@@ -5473,8 +5473,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5482,13 +5489,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5770,13 +5770,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{899DD36E-A49C-4DB8-B1CC-EB0A80891A98}">
   <dimension ref="A1:B286"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.54296875" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="26" t="s">
         <v>188</v>
       </c>
@@ -5784,1376 +5784,1376 @@
         <v>187</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="26"/>
       <c r="B2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="29"/>
       <c r="B3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="29"/>
       <c r="B4" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="24" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="24" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="24" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="24" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="24" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="25"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="23" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="24" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="24" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="24" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="24" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="24" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="25"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="23" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="24" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="25"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="25"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" s="23" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="24" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="24" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="24" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="24" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="24" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" s="24" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" s="24" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="24" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" s="25"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" s="24" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" s="24" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" s="24" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" s="24" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" s="24" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" s="24" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" s="25"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" s="24" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" s="24" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" s="24" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" s="24" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" s="24" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" s="24" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" s="24" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" s="25"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" s="23" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" s="24" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" s="24" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" s="24" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" s="24" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" s="24" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" s="24" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" s="24" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" s="25"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" s="24" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" s="24" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" s="24" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" s="24" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" s="24" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" s="25"/>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" s="24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" s="24" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" s="24" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" s="24" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" s="24" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" s="25"/>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" s="24" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" s="24" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" s="24" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" s="24" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" s="24" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" s="24" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" s="24" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" s="24" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" s="24" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A103" s="24" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A104" s="24" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" s="24" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A106" s="24" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A107" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A108" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A110" s="24" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" s="24" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" s="24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113" s="24" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A114" s="24" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A115" s="24" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A116" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A117" s="24" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A118" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A120" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A122" s="24" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" s="25"/>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" s="24" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" s="24" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A126" s="24" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A128" s="24" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A129" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A130" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A131" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" s="24" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A134" s="25"/>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" s="24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A136" s="24" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A137" s="24" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A138" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A139" s="24" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A140" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A141" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A142" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A143" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A144" s="24" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A145" s="25"/>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A146" s="24" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A147" s="24" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A148" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A149" s="24" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" s="24" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" s="24" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A152" s="24" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A153" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A154" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A156" s="24" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A157" s="25"/>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A158" s="24" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" s="24" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A160" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A161" s="24" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A162" s="24" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A163" s="24" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A164" s="24" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A165" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A166" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A167" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A168" s="24" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A169" s="25"/>
     </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A170" s="24" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A171" s="24" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A172" s="24" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A173" s="24" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A174" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A175" s="24" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A176" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A179" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" s="24" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A181" s="25"/>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" s="24" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" s="24" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184" s="24" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A185" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A186" s="24" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A187" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A188" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A190" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" s="24" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" s="25"/>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" s="24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" s="24" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195" s="24" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A196" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197" s="24" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" s="24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A199" s="24" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200" s="24" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A201" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A202" s="24" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A203" s="25"/>
     </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A204" s="24" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A205" s="24" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A206" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A207" s="24" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A208" s="24" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A209" s="24" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A210" s="24" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A211" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A212" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A213" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A214" s="24" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A215" s="25"/>
     </row>
-    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A216" s="24" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A217" s="24" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A218" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A219" s="24" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A220" s="24" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A221" s="24" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A222" s="24" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A223" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A224" s="24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A225" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A226" s="24" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A227" s="25"/>
     </row>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A228" s="23" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A229" s="24" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A230" s="24" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A231" s="24" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A232" s="24" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A233" s="24" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A234" s="24" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A235" s="24" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A236" s="24" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A237" s="24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A238" s="24" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A239" s="24" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A240" s="24" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A241" s="24" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A242" s="24" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A243" s="24" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A244" s="24" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A245" s="24" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A246" s="24" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A247" s="24" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A248" s="24" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A249" s="24" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A250" s="24" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A251" s="25"/>
     </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A252" s="23" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A253" s="24" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A254" s="24" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A255" s="24" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A256" s="24" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A257" s="24" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A258" s="24" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A259" s="24" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A260" s="24" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A261" s="24" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A262" s="25"/>
     </row>
-    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A263" s="24" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A264" s="24" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A265" s="24" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A266" s="24" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A267" s="24" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A268" s="24" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A269" s="24" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A270" s="25"/>
     </row>
-    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A271" s="13" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A272" s="25"/>
     </row>
-    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A273" s="24" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A274" s="24" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A275" s="25"/>
     </row>
-    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A276" s="24" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A277" s="24" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A278" s="24" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A279" s="24" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A280" s="24" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A281" s="24" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A282" s="24" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A283" s="24" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A284" s="25"/>
     </row>
-    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A285" s="25"/>
     </row>
-    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A286" s="13" t="s">
         <v>186</v>
       </c>
@@ -7166,17 +7166,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{972AF565-2E3F-4051-AE1C-1CCB946DA0D6}">
   <dimension ref="A1:G62"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
@@ -7187,7 +7187,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>25</v>
       </c>
@@ -7204,7 +7204,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>26</v>
       </c>
@@ -7218,13 +7218,13 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="31" t="s">
         <v>0</v>
       </c>
       <c r="C6">
@@ -7243,8 +7243,8 @@
         <v>55272</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="30"/>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="31"/>
       <c r="C7">
         <v>2</v>
       </c>
@@ -7261,8 +7261,8 @@
         <v>55272</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="30"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="31"/>
       <c r="C8">
         <v>3</v>
       </c>
@@ -7279,8 +7279,8 @@
         <v>1584.05</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="30"/>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="31"/>
       <c r="C9">
         <v>4</v>
       </c>
@@ -7297,7 +7297,7 @@
         <v>55272</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C10">
         <v>5</v>
       </c>
@@ -7314,7 +7314,7 @@
         <v>5527.75</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>2</v>
       </c>
@@ -7325,7 +7325,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>25</v>
       </c>
@@ -7342,7 +7342,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>26</v>
       </c>
@@ -7356,12 +7356,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C16">
         <v>1</v>
       </c>
@@ -7378,7 +7378,7 @@
         <v>64312.3</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C17">
         <v>2</v>
       </c>
@@ -7395,7 +7395,7 @@
         <v>64312.3</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C18">
         <v>3</v>
       </c>
@@ -7412,7 +7412,7 @@
         <v>2282.06</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C19">
         <v>4</v>
       </c>
@@ -7429,7 +7429,7 @@
         <v>64312.3</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C20">
         <v>5</v>
       </c>
@@ -7446,12 +7446,12 @@
         <v>18303.900000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C23" t="s">
         <v>25</v>
       </c>
@@ -7468,7 +7468,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C24" t="s">
         <v>26</v>
       </c>
@@ -7482,12 +7482,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C26">
         <v>1</v>
       </c>
@@ -7504,7 +7504,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C27">
         <v>2</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C28">
         <v>3</v>
       </c>
@@ -7538,7 +7538,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C29">
         <v>4</v>
       </c>
@@ -7555,7 +7555,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C30">
         <v>5</v>
       </c>
@@ -7572,12 +7572,12 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C34" t="s">
         <v>25</v>
       </c>
@@ -7594,7 +7594,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C35" t="s">
         <v>26</v>
       </c>
@@ -7608,12 +7608,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C37">
         <v>1</v>
       </c>
@@ -7630,7 +7630,7 @@
         <v>65011.4</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C38">
         <v>2</v>
       </c>
@@ -7647,7 +7647,7 @@
         <v>65011.4</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C39">
         <v>3</v>
       </c>
@@ -7664,7 +7664,7 @@
         <v>48236.1</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C40">
         <v>4</v>
       </c>
@@ -7681,7 +7681,7 @@
         <v>65011.4</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C41">
         <v>5</v>
       </c>
@@ -7698,17 +7698,17 @@
         <v>49812.6</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C45" t="s">
         <v>25</v>
       </c>
@@ -7725,7 +7725,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C46" t="s">
         <v>26</v>
       </c>
@@ -7739,12 +7739,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C48">
         <v>1</v>
       </c>
@@ -7761,7 +7761,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C49">
         <v>2</v>
       </c>
@@ -7778,7 +7778,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C50">
         <v>3</v>
       </c>
@@ -7795,7 +7795,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C51">
         <v>4</v>
       </c>
@@ -7812,7 +7812,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C52">
         <v>5</v>
       </c>
@@ -7829,7 +7829,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="14" t="s">
         <v>6</v>
       </c>
@@ -7849,7 +7849,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C56" t="s">
         <v>26</v>
       </c>
@@ -7863,12 +7863,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C58">
         <v>1</v>
       </c>
@@ -7885,7 +7885,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C59">
         <v>2</v>
       </c>
@@ -7902,7 +7902,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C60">
         <v>3</v>
       </c>
@@ -7919,7 +7919,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C61">
         <v>4</v>
       </c>
@@ -7936,7 +7936,7 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C62">
         <v>5</v>
       </c>
@@ -7964,32 +7964,32 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA28A093-846C-4F3B-8C78-08E6801904D8}">
   <dimension ref="A1:Z39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="5.140625" customWidth="1"/>
-    <col min="3" max="3" width="3.140625" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="3.85546875" customWidth="1"/>
+    <col min="2" max="2" width="5.1796875" customWidth="1"/>
+    <col min="3" max="3" width="3.1796875" customWidth="1"/>
+    <col min="4" max="4" width="17.81640625" customWidth="1"/>
+    <col min="5" max="5" width="3.81640625" customWidth="1"/>
     <col min="6" max="7" width="13" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" customWidth="1"/>
-    <col min="19" max="19" width="1.5703125" customWidth="1"/>
-    <col min="20" max="20" width="27.28515625" customWidth="1"/>
+    <col min="9" max="9" width="17.81640625" customWidth="1"/>
+    <col min="13" max="13" width="10.54296875" customWidth="1"/>
+    <col min="18" max="18" width="16.54296875" customWidth="1"/>
+    <col min="19" max="19" width="1.54296875" customWidth="1"/>
+    <col min="20" max="20" width="27.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A1" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
@@ -8009,7 +8009,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="33"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -8032,7 +8032,7 @@
         <v>6979.2790114789004</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="33"/>
       <c r="B4" s="2" t="s">
         <v>15</v>
@@ -8062,7 +8062,7 @@
         <v>1510.77542355693</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="33"/>
       <c r="B5" s="2" t="s">
         <v>16</v>
@@ -8092,7 +8092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="33"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
@@ -8118,7 +8118,7 @@
         <v>5189.5207829431502</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="33"/>
       <c r="B7" s="2" t="s">
         <v>18</v>
@@ -8144,7 +8144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="6"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -8159,7 +8159,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="33" t="s">
         <v>19</v>
       </c>
@@ -8181,7 +8181,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="33"/>
       <c r="B10" s="2" t="s">
         <v>15</v>
@@ -8211,7 +8211,7 @@
         <v>7203.9742631380104</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="33"/>
       <c r="B11" s="2" t="s">
         <v>16</v>
@@ -8241,7 +8241,7 @@
         <v>1646.9433223600499</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="33"/>
       <c r="B12" s="2" t="s">
         <v>17</v>
@@ -8267,7 +8267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="33"/>
       <c r="B13" s="2" t="s">
         <v>18</v>
@@ -8293,7 +8293,7 @@
         <v>2029.89294004658</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="33"/>
       <c r="D14" s="4">
         <f>SUM(D10:D13)</f>
@@ -8318,7 +8318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="33" t="s">
         <v>21</v>
       </c>
@@ -8338,7 +8338,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="33"/>
       <c r="B16" s="2" t="s">
         <v>15</v>
@@ -8369,16 +8369,16 @@
       <c r="M16" s="19">
         <v>16311.4</v>
       </c>
-      <c r="N16" s="35">
+      <c r="N16" s="30">
         <f>SUM(J16:M16)</f>
         <v>47754.81</v>
       </c>
-      <c r="Q16" s="31" t="s">
+      <c r="Q16" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="R16" s="32"/>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="R16" s="35"/>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17" s="33"/>
       <c r="B17" s="2" t="s">
         <v>16</v>
@@ -8420,7 +8420,7 @@
         <v>17629.87</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A18" s="33"/>
       <c r="B18" s="2" t="s">
         <v>17</v>
@@ -8458,7 +8458,7 @@
         <v>15468.46</v>
       </c>
     </row>
-    <row r="19" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="33"/>
       <c r="B19" s="2" t="s">
         <v>18</v>
@@ -8496,7 +8496,7 @@
         <v>17169.919999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A20" s="33"/>
       <c r="D20" s="4">
         <f>SUM(D16:D19)</f>
@@ -8513,12 +8513,15 @@
         <v>50268.25</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="33" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="O21">
+        <v>10115.780580721799</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A22" s="33"/>
       <c r="B22" s="2" t="s">
         <v>15</v>
@@ -8553,16 +8556,19 @@
         <f>SUM(J22:M22)</f>
         <v>45367.18</v>
       </c>
-      <c r="Q22" s="31" t="s">
+      <c r="O22">
+        <v>6443.9901154583204</v>
+      </c>
+      <c r="Q22" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="R22" s="32"/>
+      <c r="R22" s="35"/>
       <c r="S22" s="1"/>
       <c r="T22" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A23" s="33"/>
       <c r="B23" s="2" t="s">
         <v>16</v>
@@ -8597,6 +8603,9 @@
         <f t="shared" ref="N23:N25" si="1">SUM(J23:M23)</f>
         <v>44617.990000000005</v>
       </c>
+      <c r="O23">
+        <v>13997.151652852201</v>
+      </c>
       <c r="P23" s="5"/>
       <c r="Q23" s="9" t="s">
         <v>47</v>
@@ -8606,7 +8615,7 @@
       </c>
       <c r="Z23" s="17"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24" s="33"/>
       <c r="B24" s="2" t="s">
         <v>17</v>
@@ -8638,6 +8647,9 @@
         <f t="shared" si="1"/>
         <v>44338.67</v>
       </c>
+      <c r="O24">
+        <v>17197.844717036998</v>
+      </c>
       <c r="P24" s="3"/>
       <c r="Q24" s="9" t="s">
         <v>48</v>
@@ -8646,7 +8658,7 @@
         <v>13593.37</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="33"/>
       <c r="B25" s="2" t="s">
         <v>18</v>
@@ -8678,6 +8690,10 @@
         <f t="shared" si="1"/>
         <v>44756.770000000004</v>
       </c>
+      <c r="O25">
+        <f>SUM(O21:O24)</f>
+        <v>47754.767066069318</v>
+      </c>
       <c r="P25" s="3"/>
       <c r="Q25" s="10" t="s">
         <v>49</v>
@@ -8686,7 +8702,7 @@
         <v>17774.16</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26" s="33"/>
       <c r="D26" s="4">
         <f>SUM(D22:D25)</f>
@@ -8703,12 +8719,12 @@
         <v>47754.84</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A28" s="33" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A29" s="33"/>
       <c r="B29" s="2" t="s">
         <v>15</v>
@@ -8747,7 +8763,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A30" s="33"/>
       <c r="B30" s="2" t="s">
         <v>16</v>
@@ -8783,7 +8799,7 @@
         <v>47004.36</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A31" s="33"/>
       <c r="B31" s="2" t="s">
         <v>17</v>
@@ -8815,7 +8831,7 @@
         <v>46788.26</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A32" s="33"/>
       <c r="B32" s="2" t="s">
         <v>18</v>
@@ -8847,7 +8863,7 @@
         <v>46958.36</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33" s="6"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -8862,7 +8878,7 @@
       </c>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="33" t="s">
         <v>4</v>
       </c>
@@ -8870,7 +8886,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35" s="33"/>
       <c r="B35" s="2" t="s">
         <v>15</v>
@@ -8904,12 +8920,12 @@
         <f t="shared" ref="N35:N36" si="4">SUM(J35:M35)</f>
         <v>88900.200000000012</v>
       </c>
-      <c r="Q35" s="31" t="s">
+      <c r="Q35" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="R35" s="32"/>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="R35" s="35"/>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A36" s="33"/>
       <c r="B36" s="2" t="s">
         <v>16</v>
@@ -8953,7 +8969,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A37" s="33"/>
       <c r="B37" s="2" t="s">
         <v>17</v>
@@ -8993,7 +9009,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="33"/>
       <c r="B38" s="2" t="s">
         <v>18</v>
@@ -9033,7 +9049,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A39" s="33"/>
       <c r="D39" s="4">
         <f>SUM(D35:D38)</f>
@@ -9052,16 +9068,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="A21:A26"/>
+    <mergeCell ref="A34:A39"/>
+    <mergeCell ref="A28:A32"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:A7"/>
     <mergeCell ref="A9:A14"/>
     <mergeCell ref="A15:A20"/>
     <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="A21:A26"/>
-    <mergeCell ref="A34:A39"/>
-    <mergeCell ref="A28:A32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9071,18 +9087,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B691C82-6C6D-40EE-8BF2-E9DADBE04603}">
   <dimension ref="B1:Q34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="7" width="22.140625" customWidth="1"/>
+    <col min="6" max="7" width="22.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="14" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>31</v>
       </c>
@@ -9096,7 +9112,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>34</v>
       </c>
@@ -9110,7 +9126,7 @@
         <v>-503.4</v>
       </c>
     </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>36</v>
       </c>
@@ -9124,7 +9140,7 @@
         <v>-692.5</v>
       </c>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>38</v>
       </c>
@@ -9138,7 +9154,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>40</v>
       </c>
@@ -9161,7 +9177,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>40</v>
       </c>
@@ -9211,12 +9227,12 @@
         <v>198</v>
       </c>
     </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B10" s="14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>31</v>
       </c>
@@ -9230,7 +9246,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>34</v>
       </c>
@@ -9244,7 +9260,7 @@
         <v>216.4</v>
       </c>
     </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>36</v>
       </c>
@@ -9258,7 +9274,7 @@
         <v>-706</v>
       </c>
     </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>38</v>
       </c>
@@ -9272,7 +9288,7 @@
         <v>-660.5</v>
       </c>
     </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>40</v>
       </c>
@@ -9295,7 +9311,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>40</v>
       </c>
@@ -9345,12 +9361,12 @@
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B19" s="14" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>31</v>
       </c>
@@ -9364,7 +9380,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
         <v>34</v>
       </c>
@@ -9378,7 +9394,7 @@
         <v>-293.60000000000002</v>
       </c>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C22" t="s">
         <v>36</v>
       </c>
@@ -9392,7 +9408,7 @@
         <v>-1180</v>
       </c>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C23" t="s">
         <v>38</v>
       </c>
@@ -9406,7 +9422,7 @@
         <v>448.4</v>
       </c>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>40</v>
       </c>
@@ -9429,7 +9445,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>40</v>
       </c>
@@ -9479,12 +9495,12 @@
         <v>214</v>
       </c>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B28" s="14" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>31</v>
       </c>
@@ -9498,7 +9514,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C30" t="s">
         <v>34</v>
       </c>
@@ -9512,7 +9528,7 @@
         <v>157.5</v>
       </c>
     </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C31" t="s">
         <v>36</v>
       </c>
@@ -9526,7 +9542,7 @@
         <v>-471</v>
       </c>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C32" t="s">
         <v>38</v>
       </c>
@@ -9540,7 +9556,7 @@
         <v>-131.6</v>
       </c>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>40</v>
       </c>
@@ -9563,7 +9579,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>40</v>
       </c>
@@ -9621,7 +9637,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5943CADA-4813-4D4C-9452-B2A1A6727F89}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>